<commit_message>
fix: align weekly plan fills and shift legend with templates
</commit_message>
<xml_diff>
--- a/templates/Vardiyali-Calisma_Plani_10-16_Agustos.xlsx
+++ b/templates/Vardiyali-Calisma_Plani_10-16_Agustos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Puantaj_Yeni\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C575C7B1-DA8A-4193-B045-A6D718D4F3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139DB974-5916-4A4D-BBDD-3D9F5E73F249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="67">
   <si>
     <t>HAFTALIK ÇALIŞMA PLANI</t>
   </si>
@@ -165,9 +165,6 @@
     <t>HOUSMAN(JOKER)</t>
   </si>
   <si>
-    <t>1 GÜN ALAÇAK İZNİ OLAÇAK</t>
-  </si>
-  <si>
     <t>MUHAMMET ÖZBEK</t>
   </si>
   <si>
@@ -226,6 +223,9 @@
   </si>
   <si>
     <t>09/17. VARDİYASI</t>
+  </si>
+  <si>
+    <t>Comment</t>
   </si>
 </sst>
 </file>
@@ -348,17 +348,18 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="162"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -499,17 +500,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -655,58 +645,17 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -766,6 +715,52 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -777,38 +772,38 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -816,16 +811,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -835,115 +830,137 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="15" fillId="9" borderId="10" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="14" fillId="9" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="3" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1240,31 +1257,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
-      <c r="K1" s="53"/>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
-      <c r="O1" s="53"/>
-      <c r="P1" s="53"/>
-      <c r="Q1" s="53"/>
-      <c r="R1" s="53"/>
-      <c r="S1" s="54"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="61"/>
+      <c r="R1" s="61"/>
+      <c r="S1" s="62"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="55"/>
-      <c r="B2" s="55"/>
+      <c r="A2" s="63"/>
+      <c r="B2" s="63"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1284,10 +1301,10 @@
       <c r="S2" s="3"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="56"/>
+      <c r="B3" s="64"/>
       <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
@@ -1305,10 +1322,10 @@
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="57" t="s">
+      <c r="R3" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="58"/>
+      <c r="S3" s="81"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -1318,82 +1335,84 @@
       <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="59" t="s">
+      <c r="D4" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="60"/>
-      <c r="F4" s="59">
+      <c r="E4" s="52"/>
+      <c r="F4" s="51">
         <v>46245</v>
       </c>
-      <c r="G4" s="60"/>
-      <c r="H4" s="59">
+      <c r="G4" s="52"/>
+      <c r="H4" s="51">
         <v>46246</v>
       </c>
-      <c r="I4" s="60"/>
-      <c r="J4" s="59">
+      <c r="I4" s="52"/>
+      <c r="J4" s="51">
         <v>46247</v>
       </c>
-      <c r="K4" s="60"/>
-      <c r="L4" s="59">
+      <c r="K4" s="52"/>
+      <c r="L4" s="51">
         <v>46248</v>
       </c>
-      <c r="M4" s="60"/>
-      <c r="N4" s="59">
+      <c r="M4" s="52"/>
+      <c r="N4" s="51">
         <v>46249</v>
       </c>
-      <c r="O4" s="60"/>
-      <c r="P4" s="59">
+      <c r="O4" s="52"/>
+      <c r="P4" s="51">
         <v>46250</v>
       </c>
-      <c r="Q4" s="60"/>
-      <c r="R4" s="30" t="s">
+      <c r="Q4" s="52"/>
+      <c r="R4" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="S4" s="31"/>
+      <c r="S4" s="66"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="63"/>
-      <c r="B5" s="64" t="s">
+      <c r="A5" s="53"/>
+      <c r="B5" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="C5" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="66" t="s">
+      <c r="D5" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66" t="s">
+      <c r="E5" s="56"/>
+      <c r="F5" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66" t="s">
+      <c r="G5" s="56"/>
+      <c r="H5" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="66"/>
-      <c r="J5" s="66" t="s">
+      <c r="I5" s="56"/>
+      <c r="J5" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="66"/>
-      <c r="L5" s="66" t="s">
+      <c r="K5" s="56"/>
+      <c r="L5" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66" t="s">
+      <c r="M5" s="56"/>
+      <c r="N5" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66" t="s">
+      <c r="O5" s="56"/>
+      <c r="P5" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="67"/>
-      <c r="R5" s="68"/>
-      <c r="S5" s="69"/>
+      <c r="Q5" s="57"/>
+      <c r="R5" s="72" t="s">
+        <v>66</v>
+      </c>
+      <c r="S5" s="74"/>
     </row>
     <row r="6" spans="1:19" ht="24" x14ac:dyDescent="0.25">
-      <c r="A6" s="63"/>
-      <c r="B6" s="64"/>
-      <c r="C6" s="65"/>
+      <c r="A6" s="53"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="55"/>
       <c r="D6" s="6" t="s">
         <v>16</v>
       </c>
@@ -1436,16 +1455,16 @@
       <c r="Q6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="70"/>
-      <c r="S6" s="71"/>
+      <c r="R6" s="73"/>
+      <c r="S6" s="75"/>
     </row>
     <row r="7" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
-      <c r="B7" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
+      <c r="B7" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -1459,17 +1478,17 @@
       <c r="O7" s="10"/>
       <c r="P7" s="10"/>
       <c r="Q7" s="11"/>
-      <c r="R7" s="35"/>
-      <c r="S7" s="36"/>
+      <c r="R7" s="67"/>
+      <c r="S7" s="68"/>
     </row>
     <row r="8" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A8" s="37">
+      <c r="A8" s="35">
         <v>1</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="31" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="10" t="s">
@@ -1500,17 +1519,17 @@
         <v>24</v>
       </c>
       <c r="Q8" s="11"/>
-      <c r="R8" s="35"/>
-      <c r="S8" s="36"/>
+      <c r="R8" s="33"/>
+      <c r="S8" s="34"/>
     </row>
     <row r="9" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A9" s="37">
+      <c r="A9" s="35">
         <v>2</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="31" t="s">
         <v>43</v>
       </c>
       <c r="D9" s="10" t="s">
@@ -1541,28 +1560,28 @@
         <v>24</v>
       </c>
       <c r="Q9" s="11"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="36"/>
+      <c r="R9" s="33"/>
+      <c r="S9" s="34"/>
     </row>
     <row r="10" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="35">
         <v>3</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="10"/>
-      <c r="F10" s="34" t="s">
+      <c r="F10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="G10" s="10"/>
-      <c r="H10" s="34" t="s">
+      <c r="H10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="I10" s="10"/>
@@ -1570,32 +1589,30 @@
         <v>24</v>
       </c>
       <c r="K10" s="10"/>
-      <c r="L10" s="34" t="s">
+      <c r="L10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="M10" s="10"/>
-      <c r="N10" s="34" t="s">
+      <c r="N10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="O10" s="10"/>
-      <c r="P10" s="34" t="s">
+      <c r="P10" s="32" t="s">
         <v>24</v>
       </c>
       <c r="Q10" s="11"/>
-      <c r="R10" s="72" t="s">
+      <c r="R10" s="47"/>
+      <c r="S10" s="71"/>
+    </row>
+    <row r="11" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A11" s="35">
+        <v>4</v>
+      </c>
+      <c r="B11" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="S10" s="73"/>
-    </row>
-    <row r="11" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
-        <v>4</v>
-      </c>
-      <c r="B11" s="32" t="s">
+      <c r="C11" s="31" t="s">
         <v>47</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>48</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>20</v>
@@ -1625,20 +1642,20 @@
         <v>24</v>
       </c>
       <c r="Q11" s="11"/>
-      <c r="R11" s="35"/>
-      <c r="S11" s="36"/>
+      <c r="R11" s="33"/>
+      <c r="S11" s="34"/>
     </row>
     <row r="12" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A12" s="37">
+      <c r="A12" s="35">
         <v>5</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="32" t="s">
         <v>24</v>
       </c>
       <c r="E12" s="10"/>
@@ -1666,49 +1683,49 @@
         <v>24</v>
       </c>
       <c r="Q12" s="11"/>
-      <c r="R12" s="35"/>
-      <c r="S12" s="36"/>
+      <c r="R12" s="33"/>
+      <c r="S12" s="34"/>
     </row>
     <row r="13" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A13" s="37">
+      <c r="A13" s="35">
         <v>6</v>
       </c>
-      <c r="B13" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="34" t="s">
+      <c r="B13" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="J13" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="L13" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="N13" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="P13" s="34" t="s">
+      <c r="H13" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="N13" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="P13" s="32" t="s">
         <v>24</v>
       </c>
       <c r="Q13" s="11"/>
-      <c r="R13" s="35"/>
-      <c r="S13" s="36"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="34"/>
     </row>
     <row r="14" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A14" s="37"/>
-      <c r="B14" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="40"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="31"/>
+      <c r="D14" s="38"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -1722,20 +1739,20 @@
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
       <c r="Q14" s="13"/>
-      <c r="R14" s="74"/>
-      <c r="S14" s="75"/>
+      <c r="R14" s="58"/>
+      <c r="S14" s="59"/>
     </row>
     <row r="15" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A15" s="37">
+      <c r="A15" s="35">
         <v>7</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E15" s="10"/>
@@ -1763,22 +1780,20 @@
         <v>19</v>
       </c>
       <c r="Q15" s="13"/>
-      <c r="R15" s="72" t="s">
-        <v>46</v>
-      </c>
-      <c r="S15" s="73"/>
+      <c r="R15" s="47"/>
+      <c r="S15" s="71"/>
     </row>
     <row r="16" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A16" s="37">
+      <c r="A16" s="35">
         <v>8</v>
       </c>
-      <c r="B16" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="33" t="s">
+      <c r="B16" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="10"/>
@@ -1806,20 +1821,20 @@
         <v>19</v>
       </c>
       <c r="Q16" s="13"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="43"/>
+      <c r="R16" s="69"/>
+      <c r="S16" s="70"/>
     </row>
     <row r="17" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A17" s="37">
+      <c r="A17" s="35">
         <v>9</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E17" s="10"/>
@@ -1847,18 +1862,18 @@
         <v>19</v>
       </c>
       <c r="Q17" s="13"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="43"/>
+      <c r="R17" s="69"/>
+      <c r="S17" s="70"/>
     </row>
     <row r="18" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A18" s="37">
+      <c r="A18" s="35">
         <v>10</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="33" t="s">
-        <v>50</v>
+      <c r="B18" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>49</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>20</v>
@@ -1884,24 +1899,24 @@
         <v>19</v>
       </c>
       <c r="O18" s="10"/>
-      <c r="P18" s="44" t="s">
+      <c r="P18" s="40" t="s">
         <v>32</v>
       </c>
       <c r="Q18" s="13"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="43"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="70"/>
     </row>
     <row r="19" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A19" s="37">
+      <c r="A19" s="35">
         <v>11</v>
       </c>
-      <c r="B19" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="34" t="s">
+      <c r="B19" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E19" s="10"/>
@@ -1929,16 +1944,16 @@
         <v>19</v>
       </c>
       <c r="Q19" s="13"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="43"/>
+      <c r="R19" s="69"/>
+      <c r="S19" s="70"/>
     </row>
     <row r="20" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A20" s="37"/>
-      <c r="B20" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="40"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="31"/>
+      <c r="D20" s="38"/>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -1952,40 +1967,40 @@
       <c r="O20" s="12"/>
       <c r="P20" s="12"/>
       <c r="Q20" s="13"/>
-      <c r="R20" s="61"/>
-      <c r="S20" s="62"/>
+      <c r="R20" s="48"/>
+      <c r="S20" s="49"/>
     </row>
     <row r="21" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A21" s="37">
+      <c r="A21" s="35">
         <v>12</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="33" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="44" t="s">
+      <c r="D21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="E21" s="10"/>
-      <c r="F21" s="44" t="s">
+      <c r="F21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="G21" s="10"/>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="I21" s="10"/>
-      <c r="J21" s="44" t="s">
+      <c r="J21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="K21" s="10"/>
-      <c r="L21" s="44" t="s">
+      <c r="L21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="M21" s="10"/>
-      <c r="N21" s="44" t="s">
+      <c r="N21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="O21" s="10"/>
@@ -1993,18 +2008,18 @@
         <v>20</v>
       </c>
       <c r="Q21" s="13"/>
-      <c r="R21" s="72"/>
-      <c r="S21" s="73"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="71"/>
     </row>
     <row r="22" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A22" s="37">
+      <c r="A22" s="35">
         <v>13</v>
       </c>
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="31" t="s">
         <v>63</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>64</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>24</v>
@@ -2034,18 +2049,18 @@
         <v>24</v>
       </c>
       <c r="Q22" s="13"/>
-      <c r="R22" s="46"/>
-      <c r="S22" s="47"/>
+      <c r="R22" s="69"/>
+      <c r="S22" s="70"/>
     </row>
     <row r="23" spans="1:19" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A23" s="37">
+      <c r="A23" s="35">
         <v>14</v>
       </c>
-      <c r="B23" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="33" t="s">
+      <c r="B23" s="30" t="s">
         <v>64</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>63</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>24</v>
@@ -2075,29 +2090,29 @@
         <v>24</v>
       </c>
       <c r="Q23" s="13"/>
-      <c r="R23" s="61"/>
-      <c r="S23" s="62"/>
+      <c r="R23" s="48"/>
+      <c r="S23" s="49"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A24" s="48"/>
-      <c r="B24" s="49"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
       <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
       <c r="O24" s="3"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="3"/>
-      <c r="R24" s="17"/>
-      <c r="S24" s="51"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="77"/>
+      <c r="R24" s="78"/>
+      <c r="S24" s="79"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
@@ -2111,14 +2126,14 @@
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
-      <c r="K25" s="79"/>
-      <c r="L25" s="79"/>
-      <c r="M25" s="79"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
       <c r="N25" s="16"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -2138,8 +2153,8 @@
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
       <c r="H26" s="16"/>
       <c r="I26" s="16"/>
       <c r="J26" s="16"/>
@@ -2164,13 +2179,13 @@
       <c r="B27" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="77" t="s">
+      <c r="C27" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="D27" s="77"/>
-      <c r="E27" s="77"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="76"/>
+      <c r="G27" s="76"/>
       <c r="H27" s="16"/>
       <c r="I27" s="16"/>
       <c r="J27" s="16"/>
@@ -2200,14 +2215,14 @@
       </c>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
       <c r="H28" s="16"/>
       <c r="I28" s="16"/>
       <c r="J28" s="16"/>
-      <c r="K28" s="76"/>
-      <c r="L28" s="76"/>
-      <c r="M28" s="76"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
       <c r="P28" s="16"/>
@@ -2227,8 +2242,8 @@
       </c>
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
+      <c r="F29" s="76"/>
+      <c r="G29" s="76"/>
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
       <c r="J29" s="16"/>
@@ -2245,13 +2260,13 @@
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="22"/>
       <c r="B30" s="15"/>
-      <c r="C30" s="77" t="s">
+      <c r="C30" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="D30" s="77"/>
-      <c r="E30" s="77"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
+      <c r="D30" s="45"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="76"/>
+      <c r="G30" s="76"/>
       <c r="H30" s="16"/>
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
@@ -2268,11 +2283,11 @@
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="23"/>
       <c r="B31" s="3"/>
-      <c r="C31" s="78"/>
-      <c r="D31" s="78"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="76"/>
+      <c r="G31" s="76"/>
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
       <c r="J31" s="16"/>
@@ -2331,14 +2346,23 @@
       <c r="S33" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="K28:M28"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="C27:E27"/>
+  <mergeCells count="40">
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="R4:S4"/>
     <mergeCell ref="R20:S20"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="A5:A6"/>
@@ -2355,16 +2379,14 @@
     <mergeCell ref="R10:S10"/>
     <mergeCell ref="R14:S14"/>
     <mergeCell ref="R15:S15"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="R22:S22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>